<commit_message>
Created GW outputs and datetime format
</commit_message>
<xml_diff>
--- a/CWatM_settings/cwatm_settings.xlsx
+++ b/CWatM_settings/cwatm_settings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guillaumot\Documents\GitHub\FUSE\CWatM_settings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B2385E-5FDF-49D2-8F3B-F5CA5DC3A831}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11B92DF-83BB-4597-84C4-2ABE676FAD4F}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{3B47940C-5F20-42D1-80D0-733DA86DBAA8}"/>
+    <workbookView xWindow="2562" yWindow="2562" windowWidth="17280" windowHeight="8994" xr2:uid="{3B47940C-5F20-42D1-80D0-733DA86DBAA8}"/>
   </bookViews>
   <sheets>
     <sheet name="CWatM_input" sheetId="3" r:id="rId1"/>
@@ -1974,7 +1974,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2090,6 +2090,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2441,8 +2444,8 @@
       <c r="A4" s="29" t="s">
         <v>126</v>
       </c>
-      <c r="B4" s="38">
-        <v>35</v>
+      <c r="B4" s="46">
+        <v>4748</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2450,7 +2453,7 @@
         <v>407</v>
       </c>
       <c r="B5" s="39">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2">

</xml_diff>

<commit_message>
make the figures prettier for GW extraction
Created a new plots, imshow, and removed some useless plots
</commit_message>
<xml_diff>
--- a/CWatM_settings/cwatm_settings.xlsx
+++ b/CWatM_settings/cwatm_settings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guillaumot\Documents\GitHub\FUSE\CWatM_settings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11B92DF-83BB-4597-84C4-2ABE676FAD4F}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEDBA13E-AC64-4BB3-B064-B1E0E3A38A09}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2562" yWindow="2562" windowWidth="17280" windowHeight="8994" xr2:uid="{3B47940C-5F20-42D1-80D0-733DA86DBAA8}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{3B47940C-5F20-42D1-80D0-733DA86DBAA8}"/>
   </bookViews>
   <sheets>
     <sheet name="CWatM_input" sheetId="3" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="571">
   <si>
     <t>PathRoot</t>
   </si>
@@ -1737,6 +1737,15 @@
   </si>
   <si>
     <t>OUT_MAP_totalend</t>
+  </si>
+  <si>
+    <t>discharge, lakeResInflowDis, lakeResOutflowDis, lakeResStorage, act_bigLakeResAbst_alloc</t>
+  </si>
+  <si>
+    <t>0.00005</t>
+  </si>
+  <si>
+    <t>0.05</t>
   </si>
 </sst>
 </file>
@@ -2445,7 +2454,7 @@
         <v>126</v>
       </c>
       <c r="B4" s="46">
-        <v>4748</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2453,7 +2462,7 @@
         <v>407</v>
       </c>
       <c r="B5" s="39">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2468,7 +2477,9 @@
       <c r="A7" s="27" t="s">
         <v>544</v>
       </c>
-      <c r="B7" s="39"/>
+      <c r="B7" s="39" t="s">
+        <v>568</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="27" t="s">
@@ -2575,12 +2586,36 @@
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="25"/>
-      <c r="B21" s="25"/>
+      <c r="A21" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="25"/>
-      <c r="B22" s="25"/>
+      <c r="A22" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="7" t="s">
+        <v>551</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>570</v>
+      </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="25"/>

</xml_diff>

<commit_message>
Remove wells close from boundaries and modify GW criteria
</commit_message>
<xml_diff>
--- a/CWatM_settings/cwatm_settings.xlsx
+++ b/CWatM_settings/cwatm_settings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guillaumot\Documents\GitHub\FUSE\CWatM_settings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEDBA13E-AC64-4BB3-B064-B1E0E3A38A09}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3644AE-0DAC-4236-A9F0-BAA500E73048}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{3B47940C-5F20-42D1-80D0-733DA86DBAA8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="571">
   <si>
     <t>PathRoot</t>
   </si>
@@ -1715,9 +1715,6 @@
     <t xml:space="preserve"> $(FILE_PATHS:PathMaps)/init/Nira</t>
   </si>
   <si>
-    <t xml:space="preserve"> 01/01/1995</t>
-  </si>
-  <si>
     <t>modflowWaterLevel</t>
   </si>
   <si>
@@ -1742,10 +1739,13 @@
     <t>discharge, lakeResInflowDis, lakeResOutflowDis, lakeResStorage, act_bigLakeResAbst_alloc</t>
   </si>
   <si>
-    <t>0.00005</t>
-  </si>
-  <si>
     <t>0.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 01/01/1987</t>
+  </si>
+  <si>
+    <t>0.000005</t>
   </si>
 </sst>
 </file>
@@ -2438,7 +2438,7 @@
         <v>123</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>560</v>
+        <v>569</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -2454,7 +2454,7 @@
         <v>126</v>
       </c>
       <c r="B4" s="46">
-        <v>10</v>
+        <v>7665</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2462,7 +2462,7 @@
         <v>407</v>
       </c>
       <c r="B5" s="39">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2478,7 +2478,7 @@
         <v>544</v>
       </c>
       <c r="B7" s="39" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2486,7 +2486,7 @@
         <v>517</v>
       </c>
       <c r="B8" s="39" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2494,7 +2494,7 @@
         <v>100</v>
       </c>
       <c r="B9" s="42" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="14.7" thickBot="1">
@@ -2502,7 +2502,7 @@
         <v>101</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -2518,7 +2518,7 @@
         <v>117</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -2574,15 +2574,15 @@
         <v>131</v>
       </c>
       <c r="B19" s="36" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="45" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -2597,8 +2597,8 @@
       <c r="A22" s="7" t="s">
         <v>391</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>77</v>
+      <c r="B22" s="9" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -2606,7 +2606,7 @@
         <v>132</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -2614,7 +2614,7 @@
         <v>551</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="27" spans="1:2">

</xml_diff>